<commit_message>
Comparison FIELDII and PyField
</commit_message>
<xml_diff>
--- a/comparison_FIELDII/Table.xlsx
+++ b/comparison_FIELDII/Table.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\INSERM\Documents\Esteban\PyField\comparison_FIELDII\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34EE0990-A999-4CC8-8C3A-50FE8A0002D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDAB59C8-C5C7-4D87-8FD3-1F53B3BE5C3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="945" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C3599692-E6F5-48F0-8CA3-3A85ED04EF7A}"/>
   </bookViews>
@@ -735,7 +735,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -747,6 +747,100 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -759,22 +853,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -783,119 +862,38 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1264,21 +1262,21 @@
       <c r="R2" s="1"/>
     </row>
     <row r="3" spans="2:21" ht="15.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="8" t="s">
+      <c r="C3" s="37"/>
+      <c r="D3" s="40" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="40"/>
+      <c r="J3" s="40"/>
+      <c r="K3" s="40"/>
+      <c r="L3" s="40"/>
       <c r="M3" s="3" t="s">
         <v>6</v>
       </c>
@@ -1287,7 +1285,7 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
-      <c r="S3" s="8" t="s">
+      <c r="S3" s="40" t="s">
         <v>10</v>
       </c>
       <c r="U3" s="2"/>
@@ -1301,8 +1299,8 @@
         <v>20</v>
       </c>
       <c r="E4" s="3"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="7"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="39"/>
       <c r="H4" s="4"/>
       <c r="I4" s="3" t="s">
         <v>18</v>
@@ -1324,7 +1322,7 @@
         <v>9</v>
       </c>
       <c r="R4" s="3"/>
-      <c r="S4" s="8"/>
+      <c r="S4" s="40"/>
     </row>
     <row r="5" spans="2:21" ht="30" x14ac:dyDescent="0.25">
       <c r="B5" s="3" t="s">
@@ -1464,7 +1462,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA2D7288-F0D8-482C-82B3-26B0AC1B669D}">
-  <dimension ref="C5:R30"/>
+  <dimension ref="C5:Q30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="8" max="8" width="15.7109375" customWidth="1"/>
@@ -1474,597 +1472,597 @@
   </cols>
   <sheetData>
     <row r="5" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="29" t="s">
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="30" t="s">
+      <c r="I5" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="25"/>
-      <c r="K5" s="18" t="s">
+      <c r="J5" s="47"/>
+      <c r="K5" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="L5" s="18"/>
-      <c r="M5" s="30" t="s">
+      <c r="L5" s="42"/>
+      <c r="M5" s="41" t="s">
         <v>33</v>
       </c>
-      <c r="N5" s="25"/>
-      <c r="O5" s="18" t="s">
+      <c r="N5" s="47"/>
+      <c r="O5" s="42" t="s">
         <v>103</v>
       </c>
-      <c r="P5" s="18"/>
-      <c r="Q5" s="18"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
     </row>
     <row r="6" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="15" t="s">
+      <c r="E6" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="29" t="s">
+      <c r="H6" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="15" t="s">
+      <c r="I6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="29" t="s">
+      <c r="J6" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="15" t="s">
+      <c r="K6" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="15" t="s">
+      <c r="L6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="26" t="s">
+      <c r="M6" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="15" t="s">
+      <c r="N6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="O6" s="26" t="s">
+      <c r="O6" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="16" t="s">
+      <c r="P6" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="Q6" s="16" t="s">
+      <c r="Q6" s="11" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C7" s="19">
+      <c r="C7" s="12">
         <v>729</v>
       </c>
-      <c r="D7" s="12">
+      <c r="D7" s="7">
         <v>2066</v>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="7">
         <v>1280</v>
       </c>
-      <c r="F7" s="12">
+      <c r="F7" s="7">
         <v>12.812099999999999</v>
       </c>
-      <c r="G7" s="12">
+      <c r="G7" s="7">
         <v>11.2281</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="J7" s="12">
+      <c r="J7" s="7">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="K7" s="12" t="s">
+      <c r="K7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L7" s="12">
+      <c r="L7" s="7">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="M7" s="12" t="s">
+      <c r="M7" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="N7" s="12">
+      <c r="N7" s="7">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="O7" s="23">
+      <c r="O7" s="16">
         <v>6.8925000000000001</v>
       </c>
-      <c r="P7" s="23">
+      <c r="P7" s="16">
         <v>6.8474000000000004</v>
       </c>
-      <c r="Q7" s="23">
+      <c r="Q7" s="16">
         <v>6.4423000000000004</v>
       </c>
     </row>
     <row r="8" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C8" s="20">
+      <c r="C8" s="13">
         <v>68921</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="8">
         <v>2067</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="8">
         <v>1280</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="8">
         <v>12.622299999999999</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="8">
         <v>11.229699999999999</v>
       </c>
-      <c r="H8" s="13" t="s">
+      <c r="H8" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K8" s="13" t="s">
+      <c r="K8" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="L8" s="13">
+      <c r="L8" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M8" s="13" t="s">
+      <c r="M8" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="N8" s="13">
+      <c r="N8" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O8" s="22">
+      <c r="O8" s="15">
         <v>17.494399999999999</v>
       </c>
-      <c r="P8" s="22">
+      <c r="P8" s="15">
         <v>23.516999999999999</v>
       </c>
-      <c r="Q8" s="22">
+      <c r="Q8" s="15">
         <v>20.361000000000001</v>
       </c>
     </row>
     <row r="9" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C9" s="21">
+      <c r="C9" s="14">
         <v>531441</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="9">
         <v>2067</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="9">
         <v>1280</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="9">
         <v>12.599299999999999</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="9">
         <v>11.229699999999999</v>
       </c>
-      <c r="H9" s="14" t="s">
+      <c r="H9" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="I9" s="14" t="s">
+      <c r="I9" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="9">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="K9" s="14" t="s">
+      <c r="K9" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="L9" s="14">
+      <c r="L9" s="9">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="M9" s="14" t="s">
+      <c r="M9" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="N9" s="14">
+      <c r="N9" s="9">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="O9" s="24">
+      <c r="O9" s="17">
         <v>17.097300000000001</v>
       </c>
-      <c r="P9" s="24">
+      <c r="P9" s="17">
         <v>23.691400000000002</v>
       </c>
-      <c r="Q9" s="24">
+      <c r="Q9" s="17">
         <v>21.127800000000001</v>
       </c>
     </row>
     <row r="10" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C10" s="19">
+      <c r="C10" s="12">
         <v>729</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="7">
         <v>3078</v>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="7">
         <v>5120</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="8">
         <v>11.357200000000001</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="8">
         <v>9.2022999999999993</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="J10" s="12">
+      <c r="J10" s="7">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="K10" s="12" t="s">
+      <c r="K10" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="L10" s="12">
+      <c r="L10" s="7">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="M10" s="12" t="s">
+      <c r="M10" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="N10" s="12">
+      <c r="N10" s="7">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="O10" s="22">
+      <c r="O10" s="15">
         <v>9.4707000000000008</v>
       </c>
-      <c r="P10" s="22">
+      <c r="P10" s="15">
         <v>8.2152999999999992</v>
       </c>
-      <c r="Q10" s="22">
+      <c r="Q10" s="15">
         <v>11.5246</v>
       </c>
     </row>
     <row r="11" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C11" s="20">
+      <c r="C11" s="13">
         <v>68921</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="8">
         <v>3079</v>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="8">
         <v>5120</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="8">
         <v>11.249000000000001</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="8">
         <v>9.2027000000000001</v>
       </c>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="8">
         <v>3.3E-3</v>
       </c>
-      <c r="K11" s="13" t="s">
+      <c r="K11" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="L11" s="13">
+      <c r="L11" s="8">
         <v>3.3E-3</v>
       </c>
-      <c r="M11" s="13" t="s">
+      <c r="M11" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="N11" s="13">
+      <c r="N11" s="8">
         <v>3.3E-3</v>
       </c>
-      <c r="O11" s="22">
+      <c r="O11" s="15">
         <v>12.0129</v>
       </c>
-      <c r="P11" s="22">
+      <c r="P11" s="15">
         <v>16.066700000000001</v>
       </c>
-      <c r="Q11" s="22">
+      <c r="Q11" s="15">
         <v>15.8132</v>
       </c>
     </row>
     <row r="12" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C12" s="20">
+      <c r="C12" s="13">
         <v>531441</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="8">
         <v>3079</v>
       </c>
-      <c r="E12" s="13">
+      <c r="E12" s="8">
         <v>5120</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="8">
         <v>11.2362</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="8">
         <v>9.2027000000000001</v>
       </c>
-      <c r="H12" s="13" t="s">
+      <c r="H12" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="J12" s="13">
+      <c r="J12" s="8">
         <v>2.3E-3</v>
       </c>
-      <c r="K12" s="13" t="s">
+      <c r="K12" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="L12" s="13">
+      <c r="L12" s="8">
         <v>2.3E-3</v>
       </c>
-      <c r="M12" s="13" t="s">
+      <c r="M12" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="N12" s="13">
+      <c r="N12" s="8">
         <v>2.3E-3</v>
       </c>
-      <c r="O12" s="22">
+      <c r="O12" s="15">
         <v>12.2455</v>
       </c>
-      <c r="P12" s="22">
+      <c r="P12" s="15">
         <v>16.624700000000001</v>
       </c>
-      <c r="Q12" s="22">
+      <c r="Q12" s="15">
         <v>16.478200000000001</v>
       </c>
     </row>
     <row r="13" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C13" s="12">
+      <c r="C13" s="7">
         <v>68921</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="12">
         <v>1034</v>
       </c>
-      <c r="E13" s="12">
+      <c r="E13" s="7">
         <v>1280</v>
       </c>
-      <c r="F13" s="12">
+      <c r="F13" s="7">
         <v>10.2616</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="7">
         <v>9.6156000000000006</v>
       </c>
-      <c r="H13" s="12" t="s">
+      <c r="H13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="I13" s="12" t="s">
+      <c r="I13" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="7">
         <v>1.12E-2</v>
       </c>
-      <c r="K13" s="12" t="s">
+      <c r="K13" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="L13" s="12">
+      <c r="L13" s="7">
         <v>1.12E-2</v>
       </c>
-      <c r="M13" s="12" t="s">
+      <c r="M13" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="N13" s="12">
+      <c r="N13" s="7">
         <v>1.12E-2</v>
       </c>
-      <c r="O13" s="23">
+      <c r="O13" s="16">
         <v>19.515599999999999</v>
       </c>
-      <c r="P13" s="23">
+      <c r="P13" s="16">
         <v>23.357900000000001</v>
       </c>
-      <c r="Q13" s="23">
+      <c r="Q13" s="16">
         <v>23.135200000000001</v>
       </c>
     </row>
     <row r="14" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C14" s="13">
+      <c r="C14" s="8">
         <v>68921</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="13">
         <v>2067</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="8">
         <v>1280</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="8">
         <v>12.622299999999999</v>
       </c>
-      <c r="G14" s="13">
+      <c r="G14" s="8">
         <v>11.229699999999999</v>
       </c>
-      <c r="H14" s="13" t="s">
+      <c r="H14" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K14" s="13" t="s">
+      <c r="K14" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="L14" s="13">
+      <c r="L14" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M14" s="13" t="s">
+      <c r="M14" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="N14" s="13">
+      <c r="N14" s="8">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O14" s="22">
+      <c r="O14" s="15">
         <v>17.494399999999999</v>
       </c>
-      <c r="P14" s="22">
+      <c r="P14" s="15">
         <v>23.516999999999999</v>
       </c>
-      <c r="Q14" s="22">
+      <c r="Q14" s="15">
         <v>20.361000000000001</v>
       </c>
     </row>
     <row r="15" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C15" s="14">
+      <c r="C15" s="9">
         <v>68921</v>
       </c>
-      <c r="D15" s="21">
+      <c r="D15" s="14">
         <v>3100</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="9">
         <v>1280</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="9">
         <v>15.928900000000001</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="9">
         <v>12.8438</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H15" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="I15" s="14" t="s">
+      <c r="I15" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="J15" s="14">
+      <c r="J15" s="9">
         <v>3.3E-3</v>
       </c>
-      <c r="K15" s="14" t="s">
+      <c r="K15" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="L15" s="14">
+      <c r="L15" s="9">
         <v>3.3E-3</v>
       </c>
-      <c r="M15" s="14" t="s">
+      <c r="M15" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="N15" s="14">
+      <c r="N15" s="9">
         <v>3.3E-3</v>
       </c>
-      <c r="O15" s="24">
+      <c r="O15" s="17">
         <v>14.761100000000001</v>
       </c>
-      <c r="P15" s="24">
+      <c r="P15" s="17">
         <v>23.6876</v>
       </c>
-      <c r="Q15" s="24">
+      <c r="Q15" s="17">
         <v>20.753799999999998</v>
       </c>
     </row>
     <row r="16" spans="3:17" x14ac:dyDescent="0.25">
-      <c r="C16" s="12">
+      <c r="C16" s="7">
         <v>68921</v>
       </c>
-      <c r="D16" s="12">
+      <c r="D16" s="7">
         <v>2067</v>
       </c>
-      <c r="E16" s="19">
+      <c r="E16" s="12">
         <v>1280</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="8">
         <v>12.622299999999999</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="8">
         <v>11.229699999999999</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H16" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="I16" s="12" t="s">
+      <c r="I16" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="J16" s="12">
+      <c r="J16" s="7">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K16" s="12" t="s">
+      <c r="K16" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="L16" s="12">
+      <c r="L16" s="7">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M16" s="12" t="s">
+      <c r="M16" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="N16" s="12">
+      <c r="N16" s="7">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O16" s="22">
+      <c r="O16" s="15">
         <v>17.494399999999999</v>
       </c>
-      <c r="P16" s="22">
+      <c r="P16" s="15">
         <v>23.516999999999999</v>
       </c>
-      <c r="Q16" s="22">
+      <c r="Q16" s="15">
         <v>20.361000000000001</v>
       </c>
     </row>
-    <row r="17" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C17" s="14">
+    <row r="17" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C17" s="9">
         <v>68921</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="9">
         <v>2053</v>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="14">
         <v>5120</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="9">
         <v>10.2616</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="9">
         <v>8.8019999999999996</v>
       </c>
-      <c r="H17" s="14" t="s">
+      <c r="H17" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="I17" s="14" t="s">
+      <c r="I17" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="J17" s="14">
+      <c r="J17" s="9">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K17" s="14" t="s">
+      <c r="K17" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="9">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M17" s="14" t="s">
+      <c r="M17" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="N17" s="14">
+      <c r="N17" s="9">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O17" s="24">
+      <c r="O17" s="17">
         <v>12.5238</v>
       </c>
-      <c r="P17" s="24">
+      <c r="P17" s="17">
         <v>15.3864</v>
       </c>
-      <c r="Q17" s="24">
+      <c r="Q17" s="17">
         <v>15.281000000000001</v>
       </c>
     </row>
-    <row r="18" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="18" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
@@ -2081,7 +2079,7 @@
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
     </row>
-    <row r="19" spans="3:18" x14ac:dyDescent="0.25">
+    <row r="19" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -2098,501 +2096,500 @@
       <c r="P19" s="1"/>
       <c r="Q19" s="1"/>
     </row>
-    <row r="20" spans="3:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C20" s="11"/>
-      <c r="D20" s="11"/>
-      <c r="E20" s="11"/>
-      <c r="F20" s="11"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="29" t="s">
+    <row r="20" spans="3:17" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="I20" s="27" t="s">
+      <c r="I20" s="44" t="s">
         <v>31</v>
       </c>
-      <c r="J20" s="28"/>
-      <c r="K20" s="27" t="s">
+      <c r="J20" s="45"/>
+      <c r="K20" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="L20" s="28"/>
-      <c r="M20" s="27" t="s">
+      <c r="L20" s="45"/>
+      <c r="M20" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="N20" s="28"/>
-      <c r="O20" s="30" t="s">
+      <c r="N20" s="45"/>
+      <c r="O20" s="41" t="s">
         <v>103</v>
       </c>
-      <c r="P20" s="18"/>
-      <c r="Q20" s="17"/>
-    </row>
-    <row r="21" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C21" s="15" t="s">
+      <c r="P20" s="42"/>
+      <c r="Q20" s="43"/>
+    </row>
+    <row r="21" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="15" t="s">
+      <c r="F21" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="G21" s="15" t="s">
+      <c r="G21" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="H21" s="29" t="s">
+      <c r="H21" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="I21" s="26" t="s">
+      <c r="I21" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="K21" s="26" t="s">
+      <c r="K21" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="L21" s="29" t="s">
+      <c r="L21" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="M21" s="26" t="s">
+      <c r="M21" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="N21" s="29" t="s">
+      <c r="N21" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="O21" s="26" t="s">
+      <c r="O21" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="P21" s="15" t="s">
+      <c r="P21" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="Q21" s="16" t="s">
+      <c r="Q21" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="R21" s="31"/>
-    </row>
-    <row r="22" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C22" s="20">
+    </row>
+    <row r="22" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C22" s="13">
         <v>729</v>
       </c>
-      <c r="D22" s="13">
+      <c r="D22" s="8">
         <v>1485</v>
       </c>
-      <c r="E22" s="13">
+      <c r="E22" s="8">
         <v>3025</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="8">
         <v>18.060400000000001</v>
       </c>
-      <c r="G22" s="13">
+      <c r="G22" s="8">
         <v>8.9817999999999998</v>
       </c>
-      <c r="H22" s="13" t="s">
+      <c r="H22" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="8">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="K22" s="13" t="s">
+      <c r="K22" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="L22" s="13">
+      <c r="L22" s="8">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="M22" s="13" t="s">
+      <c r="M22" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="N22" s="13">
+      <c r="N22" s="8">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="O22" s="22">
+      <c r="O22" s="15">
         <v>50.677799999999998</v>
       </c>
-      <c r="P22" s="22">
+      <c r="P22" s="15">
         <v>59.511200000000002</v>
       </c>
-      <c r="Q22" s="23">
+      <c r="Q22" s="16">
         <v>79.393100000000004</v>
       </c>
     </row>
-    <row r="23" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C23" s="20">
+    <row r="23" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C23" s="13">
         <v>68921</v>
       </c>
-      <c r="D23" s="13">
+      <c r="D23" s="8">
         <v>1485</v>
       </c>
-      <c r="E23" s="13">
+      <c r="E23" s="8">
         <v>3025</v>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="8">
         <v>17.962900000000001</v>
       </c>
-      <c r="G23" s="13">
+      <c r="G23" s="8">
         <v>8.9817999999999998</v>
       </c>
-      <c r="H23" s="13" t="s">
+      <c r="H23" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="I23" s="13" t="s">
+      <c r="I23" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="J23" s="13">
+      <c r="J23" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K23" s="13" t="s">
+      <c r="K23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="L23" s="13">
+      <c r="L23" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M23" s="13" t="s">
+      <c r="M23" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="N23" s="13">
+      <c r="N23" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O23" s="22">
+      <c r="O23" s="15">
         <v>70.514099999999999</v>
       </c>
-      <c r="P23" s="22">
+      <c r="P23" s="15">
         <v>135.0719</v>
       </c>
-      <c r="Q23" s="22">
+      <c r="Q23" s="15">
         <v>133.52440000000001</v>
       </c>
     </row>
-    <row r="24" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C24" s="20">
+    <row r="24" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C24" s="13">
         <v>531441</v>
       </c>
-      <c r="D24" s="13">
+      <c r="D24" s="8">
         <v>1485</v>
       </c>
-      <c r="E24" s="13">
+      <c r="E24" s="8">
         <v>3025</v>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="8">
         <v>17.950600000000001</v>
       </c>
-      <c r="G24" s="13">
+      <c r="G24" s="8">
         <v>8.9817999999999998</v>
       </c>
-      <c r="H24" s="13" t="s">
+      <c r="H24" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K24" s="13" t="s">
+      <c r="K24" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="L24" s="13">
+      <c r="L24" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M24" s="13" t="s">
+      <c r="M24" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="N24" s="13">
+      <c r="N24" s="8">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O24" s="22">
+      <c r="O24" s="15">
         <v>68.194199999999995</v>
       </c>
-      <c r="P24" s="22">
+      <c r="P24" s="15">
         <v>132.12219999999999</v>
       </c>
-      <c r="Q24" s="22">
+      <c r="Q24" s="15">
         <v>131.08410000000001</v>
       </c>
     </row>
-    <row r="25" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C25" s="12">
+    <row r="25" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C25" s="7">
         <v>68921</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="12">
         <v>1485</v>
       </c>
-      <c r="E25" s="12">
+      <c r="E25" s="7">
         <v>3025</v>
       </c>
-      <c r="F25" s="12">
+      <c r="F25" s="7">
         <v>17.962900000000001</v>
       </c>
-      <c r="G25" s="12">
+      <c r="G25" s="7">
         <v>8.9817999999999998</v>
       </c>
-      <c r="H25" s="12" t="s">
+      <c r="H25" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="I25" s="12" t="s">
+      <c r="I25" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="J25" s="12">
+      <c r="J25" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K25" s="12" t="s">
+      <c r="K25" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="L25" s="12">
+      <c r="L25" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M25" s="12" t="s">
+      <c r="M25" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="N25" s="12">
+      <c r="N25" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O25" s="23">
+      <c r="O25" s="16">
         <v>70.514099999999999</v>
       </c>
-      <c r="P25" s="23">
+      <c r="P25" s="16">
         <v>135.0719</v>
       </c>
-      <c r="Q25" s="23">
+      <c r="Q25" s="16">
         <v>133.52440000000001</v>
       </c>
     </row>
-    <row r="26" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C26" s="13">
+    <row r="26" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C26" s="8">
         <v>68921</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="13">
         <v>2970</v>
       </c>
-      <c r="E26" s="13">
+      <c r="E26" s="8">
         <v>3025</v>
       </c>
-      <c r="F26" s="13">
+      <c r="F26" s="8">
         <v>32.449599999999997</v>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="8">
         <v>9.9635999999999996</v>
       </c>
-      <c r="H26" s="13" t="s">
+      <c r="H26" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="I26" s="13" t="s">
+      <c r="I26" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="8">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="K26" s="13" t="s">
+      <c r="K26" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="L26" s="13">
+      <c r="L26" s="8">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="M26" s="13" t="s">
+      <c r="M26" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="N26" s="13">
+      <c r="N26" s="8">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="O26" s="22">
+      <c r="O26" s="15">
         <v>49.391199999999998</v>
       </c>
-      <c r="P26" s="22">
+      <c r="P26" s="15">
         <v>134.5736</v>
       </c>
-      <c r="Q26" s="22">
+      <c r="Q26" s="15">
         <v>130.01929999999999</v>
       </c>
     </row>
-    <row r="27" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C27" s="14">
+    <row r="27" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C27" s="9">
         <v>68921</v>
       </c>
-      <c r="D27" s="21">
+      <c r="D27" s="14">
         <v>4455</v>
       </c>
-      <c r="E27" s="14">
+      <c r="E27" s="9">
         <v>3025</v>
       </c>
-      <c r="F27" s="14">
+      <c r="F27" s="9">
         <v>47.2684</v>
       </c>
-      <c r="G27" s="14">
+      <c r="G27" s="9">
         <v>10.945499999999999</v>
       </c>
-      <c r="H27" s="14" t="s">
+      <c r="H27" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="I27" s="14" t="s">
+      <c r="I27" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="J27" s="14">
+      <c r="J27" s="9">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="K27" s="14" t="s">
+      <c r="K27" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="L27" s="14">
+      <c r="L27" s="9">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="M27" s="14" t="s">
+      <c r="M27" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="N27" s="14">
+      <c r="N27" s="9">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="O27" s="24">
+      <c r="O27" s="17">
         <v>40.0443</v>
       </c>
-      <c r="P27" s="24">
+      <c r="P27" s="17">
         <v>136.0137</v>
       </c>
-      <c r="Q27" s="24">
+      <c r="Q27" s="17">
         <v>131.1095</v>
       </c>
     </row>
-    <row r="28" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C28" s="12">
+    <row r="28" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C28" s="7">
         <v>68921</v>
       </c>
-      <c r="D28" s="12">
+      <c r="D28" s="7">
         <v>1485</v>
       </c>
-      <c r="E28" s="19">
+      <c r="E28" s="12">
         <v>3025</v>
       </c>
-      <c r="F28" s="12">
+      <c r="F28" s="7">
         <v>17.962900000000001</v>
       </c>
-      <c r="G28" s="12">
+      <c r="G28" s="7">
         <v>8.9817999999999998</v>
       </c>
-      <c r="H28" s="12" t="s">
+      <c r="H28" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="I28" s="12" t="s">
+      <c r="I28" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="J28" s="12">
+      <c r="J28" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K28" s="12" t="s">
+      <c r="K28" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M28" s="12" t="s">
+      <c r="M28" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="N28" s="12">
+      <c r="N28" s="7">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O28" s="23">
+      <c r="O28" s="16">
         <v>70.514099999999999</v>
       </c>
-      <c r="P28" s="23">
+      <c r="P28" s="16">
         <v>135.0719</v>
       </c>
-      <c r="Q28" s="23">
+      <c r="Q28" s="16">
         <v>133.52440000000001</v>
       </c>
     </row>
-    <row r="29" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C29" s="13">
+    <row r="29" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C29" s="8">
         <v>68921</v>
       </c>
-      <c r="D29" s="13">
+      <c r="D29" s="8">
         <v>1471</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="13">
         <v>12100</v>
       </c>
-      <c r="F29" s="13">
+      <c r="F29" s="8">
         <v>11.5276</v>
       </c>
-      <c r="G29" s="13">
+      <c r="G29" s="8">
         <v>8.2431000000000001</v>
       </c>
-      <c r="H29" s="13" t="s">
+      <c r="H29" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="I29" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="8">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="K29" s="13" t="s">
+      <c r="K29" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="L29" s="13">
+      <c r="L29" s="8">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="M29" s="13" t="s">
+      <c r="M29" s="8" t="s">
         <v>99</v>
       </c>
-      <c r="N29" s="13">
+      <c r="N29" s="8">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="O29" s="22">
+      <c r="O29" s="15">
         <v>32.959600000000002</v>
       </c>
-      <c r="P29" s="22">
+      <c r="P29" s="15">
         <v>46.900799999999997</v>
       </c>
-      <c r="Q29" s="22">
+      <c r="Q29" s="15">
         <v>45.837000000000003</v>
       </c>
     </row>
-    <row r="30" spans="3:18" x14ac:dyDescent="0.25">
-      <c r="C30" s="14">
+    <row r="30" spans="3:17" x14ac:dyDescent="0.25">
+      <c r="C30" s="9">
         <v>68921</v>
       </c>
-      <c r="D30" s="14">
+      <c r="D30" s="9">
         <v>1467</v>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="14">
         <v>27225</v>
       </c>
-      <c r="F30" s="14">
+      <c r="F30" s="9">
         <v>10.2056</v>
       </c>
-      <c r="G30" s="14">
+      <c r="G30" s="9">
         <v>8.1077999999999992</v>
       </c>
-      <c r="H30" s="14" t="s">
+      <c r="H30" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="I30" s="14" t="s">
+      <c r="I30" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="J30" s="14">
+      <c r="J30" s="9">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="K30" s="14" t="s">
+      <c r="K30" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="L30" s="14">
+      <c r="L30" s="9">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="M30" s="14" t="s">
+      <c r="M30" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="N30" s="14">
+      <c r="N30" s="9">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="O30" s="24">
+      <c r="O30" s="17">
         <v>22.182600000000001</v>
       </c>
-      <c r="P30" s="24">
+      <c r="P30" s="17">
         <v>28.345800000000001</v>
       </c>
-      <c r="Q30" s="24">
+      <c r="Q30" s="17">
         <v>27.2742</v>
       </c>
     </row>
@@ -2940,1093 +2937,1092 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82957BD9-834E-4397-A149-C82EF3EA1A93}">
-  <dimension ref="B5:R29"/>
+  <dimension ref="B5:Q29"/>
   <sheetFormatPr defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="32"/>
-    <col min="2" max="2" width="2.7109375" style="32" customWidth="1"/>
-    <col min="3" max="7" width="6.28515625" style="32" customWidth="1"/>
-    <col min="8" max="9" width="11.7109375" style="32" customWidth="1"/>
-    <col min="10" max="10" width="6.28515625" style="32" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" style="32" customWidth="1"/>
-    <col min="12" max="12" width="6.28515625" style="32" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" style="32" customWidth="1"/>
-    <col min="14" max="14" width="6.28515625" style="32" customWidth="1"/>
-    <col min="15" max="17" width="7.7109375" style="32" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="32"/>
+    <col min="1" max="1" width="9.140625" style="20"/>
+    <col min="2" max="2" width="2.7109375" style="20" customWidth="1"/>
+    <col min="3" max="7" width="6.28515625" style="20" customWidth="1"/>
+    <col min="8" max="9" width="11.7109375" style="20" customWidth="1"/>
+    <col min="10" max="10" width="6.28515625" style="20" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" style="20" customWidth="1"/>
+    <col min="12" max="12" width="6.28515625" style="20" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" style="20" customWidth="1"/>
+    <col min="14" max="14" width="6.28515625" style="20" customWidth="1"/>
+    <col min="15" max="17" width="7.7109375" style="20" customWidth="1"/>
+    <col min="18" max="16384" width="9.140625" style="20"/>
   </cols>
   <sheetData>
     <row r="5" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35" t="s">
+      <c r="C5" s="51"/>
+      <c r="D5" s="51"/>
+      <c r="E5" s="51"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="I5" s="36" t="s">
+      <c r="I5" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="37"/>
-      <c r="K5" s="38" t="s">
+      <c r="J5" s="53"/>
+      <c r="K5" s="54" t="s">
         <v>32</v>
       </c>
-      <c r="L5" s="38"/>
-      <c r="M5" s="36" t="s">
+      <c r="L5" s="54"/>
+      <c r="M5" s="52" t="s">
         <v>33</v>
       </c>
-      <c r="N5" s="37"/>
-      <c r="O5" s="38" t="s">
+      <c r="N5" s="53"/>
+      <c r="O5" s="54" t="s">
         <v>103</v>
       </c>
-      <c r="P5" s="38"/>
-      <c r="Q5" s="38"/>
+      <c r="P5" s="54"/>
+      <c r="Q5" s="54"/>
     </row>
     <row r="6" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="39" t="s">
+      <c r="D6" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="39" t="s">
+      <c r="E6" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="39" t="s">
+      <c r="F6" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="G6" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="35" t="s">
+      <c r="H6" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="39" t="s">
+      <c r="I6" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="35" t="s">
+      <c r="J6" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="39" t="s">
+      <c r="K6" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="39" t="s">
+      <c r="L6" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="M6" s="41" t="s">
+      <c r="M6" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="N6" s="39" t="s">
+      <c r="N6" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="O6" s="41" t="s">
+      <c r="O6" s="23" t="s">
         <v>46</v>
       </c>
-      <c r="P6" s="40" t="s">
+      <c r="P6" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="Q6" s="40" t="s">
+      <c r="Q6" s="25" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="7" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="C7" s="42">
+      <c r="C7" s="26">
         <v>729</v>
       </c>
-      <c r="D7" s="43">
+      <c r="D7" s="27">
         <v>2066</v>
       </c>
-      <c r="E7" s="43">
+      <c r="E7" s="27">
         <v>1280</v>
       </c>
-      <c r="F7" s="44">
+      <c r="F7" s="28">
         <v>12.81</v>
       </c>
-      <c r="G7" s="44">
+      <c r="G7" s="28">
         <v>11.23</v>
       </c>
-      <c r="H7" s="43" t="s">
+      <c r="H7" s="27" t="s">
         <v>135</v>
       </c>
-      <c r="I7" s="43" t="s">
+      <c r="I7" s="27" t="s">
         <v>136</v>
       </c>
-      <c r="J7" s="43">
+      <c r="J7" s="27">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="K7" s="43" t="s">
+      <c r="K7" s="27" t="s">
         <v>137</v>
       </c>
-      <c r="L7" s="43">
+      <c r="L7" s="27">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="M7" s="43" t="s">
+      <c r="M7" s="27" t="s">
         <v>138</v>
       </c>
-      <c r="N7" s="43">
+      <c r="N7" s="27">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="O7" s="44">
+      <c r="O7" s="28">
         <v>6.89</v>
       </c>
-      <c r="P7" s="44">
+      <c r="P7" s="28">
         <v>6.85</v>
       </c>
-      <c r="Q7" s="44">
+      <c r="Q7" s="28">
         <v>6.44</v>
       </c>
     </row>
     <row r="8" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="52"/>
-      <c r="C8" s="45">
+      <c r="B8" s="49"/>
+      <c r="C8" s="29">
         <v>68921</v>
       </c>
-      <c r="D8" s="46">
+      <c r="D8" s="30">
         <v>2067</v>
       </c>
-      <c r="E8" s="46">
+      <c r="E8" s="30">
         <v>1280</v>
       </c>
-      <c r="F8" s="47">
+      <c r="F8" s="31">
         <v>12.62</v>
       </c>
-      <c r="G8" s="47">
+      <c r="G8" s="31">
         <v>11.23</v>
       </c>
-      <c r="H8" s="46" t="s">
+      <c r="H8" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="I8" s="46" t="s">
+      <c r="I8" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="J8" s="46">
+      <c r="J8" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K8" s="46" t="s">
+      <c r="K8" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="L8" s="46">
+      <c r="L8" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M8" s="46" t="s">
+      <c r="M8" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="N8" s="46">
+      <c r="N8" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O8" s="47">
+      <c r="O8" s="31">
         <v>17.489999999999998</v>
       </c>
-      <c r="P8" s="47">
+      <c r="P8" s="31">
         <v>23.52</v>
       </c>
-      <c r="Q8" s="47">
+      <c r="Q8" s="31">
         <v>20.36</v>
       </c>
     </row>
     <row r="9" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="52"/>
-      <c r="C9" s="48">
+      <c r="B9" s="49"/>
+      <c r="C9" s="32">
         <v>531441</v>
       </c>
-      <c r="D9" s="49">
+      <c r="D9" s="33">
         <v>2067</v>
       </c>
-      <c r="E9" s="49">
+      <c r="E9" s="33">
         <v>1280</v>
       </c>
-      <c r="F9" s="50">
+      <c r="F9" s="34">
         <v>12.6</v>
       </c>
-      <c r="G9" s="50">
+      <c r="G9" s="34">
         <v>11.23</v>
       </c>
-      <c r="H9" s="49" t="s">
+      <c r="H9" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="I9" s="49" t="s">
+      <c r="I9" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="J9" s="49">
+      <c r="J9" s="33">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="K9" s="49" t="s">
+      <c r="K9" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="L9" s="49">
+      <c r="L9" s="33">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="M9" s="49" t="s">
+      <c r="M9" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="N9" s="49">
+      <c r="N9" s="33">
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="O9" s="50">
+      <c r="O9" s="34">
         <v>17.100000000000001</v>
       </c>
-      <c r="P9" s="50">
+      <c r="P9" s="34">
         <v>23.69</v>
       </c>
-      <c r="Q9" s="50">
+      <c r="Q9" s="34">
         <v>21.13</v>
       </c>
     </row>
     <row r="10" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="52"/>
-      <c r="C10" s="42">
+      <c r="B10" s="49"/>
+      <c r="C10" s="26">
         <v>729</v>
       </c>
-      <c r="D10" s="43">
+      <c r="D10" s="27">
         <v>3078</v>
       </c>
-      <c r="E10" s="43">
+      <c r="E10" s="27">
         <v>5120</v>
       </c>
-      <c r="F10" s="47">
+      <c r="F10" s="31">
         <v>11.36</v>
       </c>
-      <c r="G10" s="47">
+      <c r="G10" s="31">
         <v>9.1999999999999993</v>
       </c>
-      <c r="H10" s="43" t="s">
+      <c r="H10" s="27" t="s">
         <v>147</v>
       </c>
-      <c r="I10" s="43" t="s">
+      <c r="I10" s="27" t="s">
         <v>148</v>
       </c>
-      <c r="J10" s="43">
+      <c r="J10" s="27">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="K10" s="43" t="s">
+      <c r="K10" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="L10" s="43">
+      <c r="L10" s="27">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="M10" s="43" t="s">
+      <c r="M10" s="27" t="s">
         <v>150</v>
       </c>
-      <c r="N10" s="43">
+      <c r="N10" s="27">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="O10" s="47">
+      <c r="O10" s="31">
         <v>9.4700000000000006</v>
       </c>
-      <c r="P10" s="47">
+      <c r="P10" s="31">
         <v>8.2200000000000006</v>
       </c>
-      <c r="Q10" s="47">
+      <c r="Q10" s="31">
         <v>11.52</v>
       </c>
     </row>
     <row r="11" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="52"/>
-      <c r="C11" s="45">
+      <c r="B11" s="49"/>
+      <c r="C11" s="29">
         <v>68921</v>
       </c>
-      <c r="D11" s="46">
+      <c r="D11" s="30">
         <v>3079</v>
       </c>
-      <c r="E11" s="46">
+      <c r="E11" s="30">
         <v>5120</v>
       </c>
-      <c r="F11" s="47">
+      <c r="F11" s="31">
         <v>11.25</v>
       </c>
-      <c r="G11" s="47">
+      <c r="G11" s="31">
         <v>9.1999999999999993</v>
       </c>
-      <c r="H11" s="46" t="s">
+      <c r="H11" s="30" t="s">
         <v>151</v>
       </c>
-      <c r="I11" s="46" t="s">
+      <c r="I11" s="30" t="s">
         <v>152</v>
       </c>
-      <c r="J11" s="46">
+      <c r="J11" s="30">
         <v>3.3E-3</v>
       </c>
-      <c r="K11" s="46" t="s">
+      <c r="K11" s="30" t="s">
         <v>153</v>
       </c>
-      <c r="L11" s="46">
+      <c r="L11" s="30">
         <v>3.3E-3</v>
       </c>
-      <c r="M11" s="46" t="s">
+      <c r="M11" s="30" t="s">
         <v>154</v>
       </c>
-      <c r="N11" s="46">
+      <c r="N11" s="30">
         <v>3.3E-3</v>
       </c>
-      <c r="O11" s="47">
+      <c r="O11" s="31">
         <v>12.01</v>
       </c>
-      <c r="P11" s="47">
+      <c r="P11" s="31">
         <v>16.07</v>
       </c>
-      <c r="Q11" s="47">
+      <c r="Q11" s="31">
         <v>15.81</v>
       </c>
     </row>
     <row r="12" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="52"/>
-      <c r="C12" s="45">
+      <c r="B12" s="49"/>
+      <c r="C12" s="29">
         <v>531441</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="30">
         <v>3079</v>
       </c>
-      <c r="E12" s="46">
+      <c r="E12" s="30">
         <v>5120</v>
       </c>
-      <c r="F12" s="47">
+      <c r="F12" s="31">
         <v>11.24</v>
       </c>
-      <c r="G12" s="47">
+      <c r="G12" s="31">
         <v>9.1999999999999993</v>
       </c>
-      <c r="H12" s="46" t="s">
+      <c r="H12" s="30" t="s">
         <v>155</v>
       </c>
-      <c r="I12" s="46" t="s">
+      <c r="I12" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="J12" s="46">
+      <c r="J12" s="30">
         <v>2.3E-3</v>
       </c>
-      <c r="K12" s="46" t="s">
+      <c r="K12" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="L12" s="46">
+      <c r="L12" s="30">
         <v>2.3E-3</v>
       </c>
-      <c r="M12" s="46" t="s">
+      <c r="M12" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="N12" s="46">
+      <c r="N12" s="30">
         <v>2.3E-3</v>
       </c>
-      <c r="O12" s="47">
+      <c r="O12" s="31">
         <v>12.25</v>
       </c>
-      <c r="P12" s="47">
+      <c r="P12" s="31">
         <v>16.62</v>
       </c>
-      <c r="Q12" s="47">
+      <c r="Q12" s="31">
         <v>16.48</v>
       </c>
     </row>
     <row r="13" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="52"/>
-      <c r="C13" s="43">
+      <c r="B13" s="49"/>
+      <c r="C13" s="27">
         <v>68921</v>
       </c>
-      <c r="D13" s="42">
+      <c r="D13" s="26">
         <v>1034</v>
       </c>
-      <c r="E13" s="43">
+      <c r="E13" s="27">
         <v>1280</v>
       </c>
-      <c r="F13" s="44">
+      <c r="F13" s="28">
         <v>10.26</v>
       </c>
-      <c r="G13" s="44">
+      <c r="G13" s="28">
         <v>9.6199999999999992</v>
       </c>
-      <c r="H13" s="43" t="s">
+      <c r="H13" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="I13" s="43" t="s">
+      <c r="I13" s="27" t="s">
         <v>160</v>
       </c>
-      <c r="J13" s="43">
+      <c r="J13" s="27">
         <v>1.12E-2</v>
       </c>
-      <c r="K13" s="43" t="s">
+      <c r="K13" s="27" t="s">
         <v>161</v>
       </c>
-      <c r="L13" s="43">
+      <c r="L13" s="27">
         <v>1.12E-2</v>
       </c>
-      <c r="M13" s="43" t="s">
+      <c r="M13" s="27" t="s">
         <v>162</v>
       </c>
-      <c r="N13" s="43">
+      <c r="N13" s="27">
         <v>1.12E-2</v>
       </c>
-      <c r="O13" s="44">
+      <c r="O13" s="28">
         <v>19.52</v>
       </c>
-      <c r="P13" s="44">
+      <c r="P13" s="28">
         <v>23.36</v>
       </c>
-      <c r="Q13" s="44">
+      <c r="Q13" s="28">
         <v>23.14</v>
       </c>
     </row>
     <row r="14" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="52"/>
-      <c r="C14" s="46">
+      <c r="B14" s="49"/>
+      <c r="C14" s="30">
         <v>68921</v>
       </c>
-      <c r="D14" s="45">
+      <c r="D14" s="29">
         <v>2067</v>
       </c>
-      <c r="E14" s="46">
+      <c r="E14" s="30">
         <v>1280</v>
       </c>
-      <c r="F14" s="47">
+      <c r="F14" s="31">
         <v>12.62</v>
       </c>
-      <c r="G14" s="47">
+      <c r="G14" s="31">
         <v>11.23</v>
       </c>
-      <c r="H14" s="46" t="s">
+      <c r="H14" s="30" t="s">
         <v>139</v>
       </c>
-      <c r="I14" s="46" t="s">
+      <c r="I14" s="30" t="s">
         <v>140</v>
       </c>
-      <c r="J14" s="46">
+      <c r="J14" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K14" s="46" t="s">
+      <c r="K14" s="30" t="s">
         <v>141</v>
       </c>
-      <c r="L14" s="46">
+      <c r="L14" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M14" s="46" t="s">
+      <c r="M14" s="30" t="s">
         <v>142</v>
       </c>
-      <c r="N14" s="46">
+      <c r="N14" s="30">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O14" s="47">
+      <c r="O14" s="31">
         <v>17.489999999999998</v>
       </c>
-      <c r="P14" s="47">
+      <c r="P14" s="31">
         <v>23.52</v>
       </c>
-      <c r="Q14" s="47">
+      <c r="Q14" s="31">
         <v>20.36</v>
       </c>
     </row>
     <row r="15" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="52"/>
-      <c r="C15" s="49">
+      <c r="B15" s="49"/>
+      <c r="C15" s="33">
         <v>68921</v>
       </c>
-      <c r="D15" s="48">
+      <c r="D15" s="32">
         <v>3100</v>
       </c>
-      <c r="E15" s="49">
+      <c r="E15" s="33">
         <v>1280</v>
       </c>
-      <c r="F15" s="50">
+      <c r="F15" s="34">
         <v>15.93</v>
       </c>
-      <c r="G15" s="50">
+      <c r="G15" s="34">
         <v>12.84</v>
       </c>
-      <c r="H15" s="49" t="s">
+      <c r="H15" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="I15" s="49" t="s">
+      <c r="I15" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="J15" s="49">
+      <c r="J15" s="33">
         <v>3.3E-3</v>
       </c>
-      <c r="K15" s="49" t="s">
+      <c r="K15" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="L15" s="49">
+      <c r="L15" s="33">
         <v>3.3E-3</v>
       </c>
-      <c r="M15" s="49" t="s">
+      <c r="M15" s="33" t="s">
         <v>166</v>
       </c>
-      <c r="N15" s="49">
+      <c r="N15" s="33">
         <v>3.3E-3</v>
       </c>
-      <c r="O15" s="50">
+      <c r="O15" s="34">
         <v>14.76</v>
       </c>
-      <c r="P15" s="50">
+      <c r="P15" s="34">
         <v>23.69</v>
       </c>
-      <c r="Q15" s="50">
+      <c r="Q15" s="34">
         <v>20.75</v>
       </c>
     </row>
     <row r="16" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="52"/>
-      <c r="C16" s="43">
+      <c r="B16" s="49"/>
+      <c r="C16" s="27">
         <v>68921</v>
       </c>
-      <c r="D16" s="43">
+      <c r="D16" s="27">
         <v>2067</v>
       </c>
-      <c r="E16" s="42">
+      <c r="E16" s="26">
         <v>1280</v>
       </c>
-      <c r="F16" s="47">
+      <c r="F16" s="31">
         <v>12.62</v>
       </c>
-      <c r="G16" s="47">
+      <c r="G16" s="31">
         <v>11.23</v>
       </c>
-      <c r="H16" s="43" t="s">
+      <c r="H16" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="I16" s="43" t="s">
+      <c r="I16" s="27" t="s">
         <v>140</v>
       </c>
-      <c r="J16" s="43">
+      <c r="J16" s="27">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="K16" s="43" t="s">
+      <c r="K16" s="27" t="s">
         <v>141</v>
       </c>
-      <c r="L16" s="43">
+      <c r="L16" s="27">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="M16" s="43" t="s">
+      <c r="M16" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="N16" s="43">
+      <c r="N16" s="27">
         <v>3.7000000000000002E-3</v>
       </c>
-      <c r="O16" s="47">
+      <c r="O16" s="31">
         <v>17.489999999999998</v>
       </c>
-      <c r="P16" s="47">
+      <c r="P16" s="31">
         <v>23.52</v>
       </c>
-      <c r="Q16" s="47">
+      <c r="Q16" s="31">
         <v>20.36</v>
       </c>
     </row>
-    <row r="17" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="53"/>
-      <c r="C17" s="46">
+    <row r="17" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="50"/>
+      <c r="C17" s="30">
         <v>68921</v>
       </c>
-      <c r="D17" s="46">
+      <c r="D17" s="30">
         <v>2053</v>
       </c>
-      <c r="E17" s="45">
+      <c r="E17" s="29">
         <v>5120</v>
       </c>
-      <c r="F17" s="47">
+      <c r="F17" s="31">
         <v>10.26</v>
       </c>
-      <c r="G17" s="47">
+      <c r="G17" s="31">
         <v>8.8000000000000007</v>
       </c>
-      <c r="H17" s="46" t="s">
+      <c r="H17" s="30" t="s">
         <v>167</v>
       </c>
-      <c r="I17" s="46" t="s">
+      <c r="I17" s="30" t="s">
         <v>168</v>
       </c>
-      <c r="J17" s="46">
+      <c r="J17" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K17" s="46" t="s">
+      <c r="K17" s="30" t="s">
         <v>169</v>
       </c>
-      <c r="L17" s="46">
+      <c r="L17" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M17" s="46" t="s">
+      <c r="M17" s="30" t="s">
         <v>170</v>
       </c>
-      <c r="N17" s="46">
+      <c r="N17" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O17" s="47">
+      <c r="O17" s="31">
         <v>12.52</v>
       </c>
-      <c r="P17" s="47">
+      <c r="P17" s="31">
         <v>15.39</v>
       </c>
-      <c r="Q17" s="47">
+      <c r="Q17" s="31">
         <v>15.28</v>
       </c>
     </row>
-    <row r="18" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C18" s="39"/>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
-      <c r="H18" s="39"/>
-      <c r="I18" s="39"/>
-      <c r="J18" s="39"/>
-      <c r="K18" s="39"/>
-      <c r="L18" s="39"/>
-      <c r="M18" s="39"/>
-      <c r="N18" s="39"/>
-      <c r="O18" s="39"/>
-      <c r="P18" s="39"/>
-      <c r="Q18" s="39"/>
-    </row>
-    <row r="19" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="51" t="s">
+    <row r="18" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="35"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="24"/>
+      <c r="I18" s="24"/>
+      <c r="J18" s="24"/>
+      <c r="K18" s="24"/>
+      <c r="L18" s="24"/>
+      <c r="M18" s="24"/>
+      <c r="N18" s="24"/>
+      <c r="O18" s="24"/>
+      <c r="P18" s="24"/>
+      <c r="Q18" s="24"/>
+    </row>
+    <row r="19" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="48" t="s">
         <v>105</v>
       </c>
-      <c r="C19" s="45">
+      <c r="C19" s="29">
         <v>729</v>
       </c>
-      <c r="D19" s="46">
+      <c r="D19" s="30">
         <v>1485</v>
       </c>
-      <c r="E19" s="46">
+      <c r="E19" s="30">
         <v>3025</v>
       </c>
-      <c r="F19" s="47">
+      <c r="F19" s="31">
         <v>18.059999999999999</v>
       </c>
-      <c r="G19" s="47">
+      <c r="G19" s="31">
         <v>8.98</v>
       </c>
-      <c r="H19" s="46" t="s">
+      <c r="H19" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="I19" s="46" t="s">
+      <c r="I19" s="30" t="s">
         <v>108</v>
       </c>
-      <c r="J19" s="46">
+      <c r="J19" s="30">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="K19" s="46" t="s">
+      <c r="K19" s="30" t="s">
         <v>109</v>
       </c>
-      <c r="L19" s="46">
+      <c r="L19" s="30">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="M19" s="46" t="s">
+      <c r="M19" s="30" t="s">
         <v>110</v>
       </c>
-      <c r="N19" s="46">
+      <c r="N19" s="30">
         <v>7.7000000000000002E-3</v>
       </c>
-      <c r="O19" s="47">
+      <c r="O19" s="31">
         <v>50.68</v>
       </c>
-      <c r="P19" s="47">
+      <c r="P19" s="31">
         <v>59.51</v>
       </c>
-      <c r="Q19" s="47">
+      <c r="Q19" s="31">
         <v>79.39</v>
       </c>
     </row>
-    <row r="20" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="52"/>
-      <c r="C20" s="45">
+    <row r="20" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="49"/>
+      <c r="C20" s="29">
         <v>68921</v>
       </c>
-      <c r="D20" s="46">
+      <c r="D20" s="30">
         <v>1485</v>
       </c>
-      <c r="E20" s="46">
+      <c r="E20" s="30">
         <v>3025</v>
       </c>
-      <c r="F20" s="47">
+      <c r="F20" s="31">
         <v>17.96</v>
       </c>
-      <c r="G20" s="47">
+      <c r="G20" s="31">
         <v>8.98</v>
       </c>
-      <c r="H20" s="46" t="s">
+      <c r="H20" s="30" t="s">
         <v>111</v>
       </c>
-      <c r="I20" s="46" t="s">
+      <c r="I20" s="30" t="s">
         <v>112</v>
       </c>
-      <c r="J20" s="46">
+      <c r="J20" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K20" s="46" t="s">
+      <c r="K20" s="30" t="s">
         <v>113</v>
       </c>
-      <c r="L20" s="46">
+      <c r="L20" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M20" s="46" t="s">
+      <c r="M20" s="30" t="s">
         <v>114</v>
       </c>
-      <c r="N20" s="46">
+      <c r="N20" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O20" s="47">
+      <c r="O20" s="31">
         <v>70.510000000000005</v>
       </c>
-      <c r="P20" s="47">
+      <c r="P20" s="31">
         <v>135.07</v>
       </c>
-      <c r="Q20" s="47">
+      <c r="Q20" s="31">
         <v>133.52000000000001</v>
       </c>
     </row>
-    <row r="21" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="52"/>
-      <c r="C21" s="45">
+    <row r="21" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="49"/>
+      <c r="C21" s="29">
         <v>531441</v>
       </c>
-      <c r="D21" s="46">
+      <c r="D21" s="30">
         <v>1485</v>
       </c>
-      <c r="E21" s="46">
+      <c r="E21" s="30">
         <v>3025</v>
       </c>
-      <c r="F21" s="47">
+      <c r="F21" s="31">
         <v>17.95</v>
       </c>
-      <c r="G21" s="47">
+      <c r="G21" s="31">
         <v>8.98</v>
       </c>
-      <c r="H21" s="46" t="s">
+      <c r="H21" s="30" t="s">
         <v>115</v>
       </c>
-      <c r="I21" s="46" t="s">
+      <c r="I21" s="30" t="s">
         <v>116</v>
       </c>
-      <c r="J21" s="46">
+      <c r="J21" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K21" s="46" t="s">
+      <c r="K21" s="30" t="s">
         <v>117</v>
       </c>
-      <c r="L21" s="46">
+      <c r="L21" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M21" s="46" t="s">
+      <c r="M21" s="30" t="s">
         <v>118</v>
       </c>
-      <c r="N21" s="46">
+      <c r="N21" s="30">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O21" s="47">
+      <c r="O21" s="31">
         <v>68.19</v>
       </c>
-      <c r="P21" s="47">
+      <c r="P21" s="31">
         <v>132.12</v>
       </c>
-      <c r="Q21" s="47">
+      <c r="Q21" s="31">
         <v>131.08000000000001</v>
       </c>
-      <c r="R21" s="55"/>
-    </row>
-    <row r="22" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="52"/>
-      <c r="C22" s="43">
+    </row>
+    <row r="22" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="49"/>
+      <c r="C22" s="27">
         <v>68921</v>
       </c>
-      <c r="D22" s="42">
+      <c r="D22" s="26">
         <v>1485</v>
       </c>
-      <c r="E22" s="43">
+      <c r="E22" s="27">
         <v>3025</v>
       </c>
-      <c r="F22" s="44">
+      <c r="F22" s="28">
         <v>17.96</v>
       </c>
-      <c r="G22" s="44">
+      <c r="G22" s="28">
         <v>8.98</v>
       </c>
-      <c r="H22" s="43" t="s">
+      <c r="H22" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="I22" s="43" t="s">
+      <c r="I22" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="J22" s="43">
+      <c r="J22" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K22" s="43" t="s">
+      <c r="K22" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="L22" s="43">
+      <c r="L22" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M22" s="43" t="s">
+      <c r="M22" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="N22" s="43">
+      <c r="N22" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O22" s="44">
+      <c r="O22" s="28">
         <v>70.510000000000005</v>
       </c>
-      <c r="P22" s="44">
+      <c r="P22" s="28">
         <v>135.07</v>
       </c>
-      <c r="Q22" s="44">
+      <c r="Q22" s="28">
         <v>133.52000000000001</v>
       </c>
     </row>
-    <row r="23" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="52"/>
-      <c r="C23" s="46">
+    <row r="23" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="49"/>
+      <c r="C23" s="30">
         <v>68921</v>
       </c>
-      <c r="D23" s="45">
+      <c r="D23" s="29">
         <v>2970</v>
       </c>
-      <c r="E23" s="46">
+      <c r="E23" s="30">
         <v>3025</v>
       </c>
-      <c r="F23" s="47">
+      <c r="F23" s="31">
         <v>32.450000000000003</v>
       </c>
-      <c r="G23" s="47">
+      <c r="G23" s="31">
         <v>9.9600000000000009</v>
       </c>
-      <c r="H23" s="46" t="s">
+      <c r="H23" s="30" t="s">
         <v>119</v>
       </c>
-      <c r="I23" s="46" t="s">
+      <c r="I23" s="30" t="s">
         <v>120</v>
       </c>
-      <c r="J23" s="46">
+      <c r="J23" s="30">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="K23" s="46" t="s">
+      <c r="K23" s="30" t="s">
         <v>121</v>
       </c>
-      <c r="L23" s="46">
+      <c r="L23" s="30">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="M23" s="46" t="s">
+      <c r="M23" s="30" t="s">
         <v>122</v>
       </c>
-      <c r="N23" s="46">
+      <c r="N23" s="30">
         <v>8.9999999999999998E-4</v>
       </c>
-      <c r="O23" s="47">
+      <c r="O23" s="31">
         <v>49.39</v>
       </c>
-      <c r="P23" s="47">
+      <c r="P23" s="31">
         <v>134.57</v>
       </c>
-      <c r="Q23" s="47">
+      <c r="Q23" s="31">
         <v>130.02000000000001</v>
       </c>
     </row>
-    <row r="24" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="52"/>
-      <c r="C24" s="49">
+    <row r="24" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="49"/>
+      <c r="C24" s="33">
         <v>68921</v>
       </c>
-      <c r="D24" s="48">
+      <c r="D24" s="32">
         <v>4455</v>
       </c>
-      <c r="E24" s="49">
+      <c r="E24" s="33">
         <v>3025</v>
       </c>
-      <c r="F24" s="50">
+      <c r="F24" s="34">
         <v>47.27</v>
       </c>
-      <c r="G24" s="50">
+      <c r="G24" s="34">
         <v>10.95</v>
       </c>
-      <c r="H24" s="49" t="s">
+      <c r="H24" s="33" t="s">
         <v>123</v>
       </c>
-      <c r="I24" s="49" t="s">
+      <c r="I24" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="J24" s="49">
+      <c r="J24" s="33">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="K24" s="49" t="s">
+      <c r="K24" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="L24" s="49">
+      <c r="L24" s="33">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="M24" s="49" t="s">
+      <c r="M24" s="33" t="s">
         <v>126</v>
       </c>
-      <c r="N24" s="49">
+      <c r="N24" s="33">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="O24" s="50">
+      <c r="O24" s="34">
         <v>40.04</v>
       </c>
-      <c r="P24" s="50">
+      <c r="P24" s="34">
         <v>136.01</v>
       </c>
-      <c r="Q24" s="50">
+      <c r="Q24" s="34">
         <v>131.11000000000001</v>
       </c>
     </row>
-    <row r="25" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="52"/>
-      <c r="C25" s="43">
+    <row r="25" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="49"/>
+      <c r="C25" s="27">
         <v>68921</v>
       </c>
-      <c r="D25" s="43">
+      <c r="D25" s="27">
         <v>1485</v>
       </c>
-      <c r="E25" s="42">
+      <c r="E25" s="26">
         <v>3025</v>
       </c>
-      <c r="F25" s="44">
+      <c r="F25" s="28">
         <v>17.96</v>
       </c>
-      <c r="G25" s="44">
+      <c r="G25" s="28">
         <v>8.98</v>
       </c>
-      <c r="H25" s="43" t="s">
+      <c r="H25" s="27" t="s">
         <v>111</v>
       </c>
-      <c r="I25" s="43" t="s">
+      <c r="I25" s="27" t="s">
         <v>112</v>
       </c>
-      <c r="J25" s="43">
+      <c r="J25" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="K25" s="43" t="s">
+      <c r="K25" s="27" t="s">
         <v>113</v>
       </c>
-      <c r="L25" s="43">
+      <c r="L25" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="M25" s="43" t="s">
+      <c r="M25" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="N25" s="43">
+      <c r="N25" s="27">
         <v>3.5000000000000001E-3</v>
       </c>
-      <c r="O25" s="44">
+      <c r="O25" s="28">
         <v>70.510000000000005</v>
       </c>
-      <c r="P25" s="44">
+      <c r="P25" s="28">
         <v>135.07</v>
       </c>
-      <c r="Q25" s="44">
+      <c r="Q25" s="28">
         <v>133.52000000000001</v>
       </c>
     </row>
-    <row r="26" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="52"/>
-      <c r="C26" s="46">
+    <row r="26" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="49"/>
+      <c r="C26" s="30">
         <v>68921</v>
       </c>
-      <c r="D26" s="46">
+      <c r="D26" s="30">
         <v>1471</v>
       </c>
-      <c r="E26" s="45">
+      <c r="E26" s="29">
         <v>12100</v>
       </c>
-      <c r="F26" s="47">
+      <c r="F26" s="31">
         <v>11.53</v>
       </c>
-      <c r="G26" s="47">
+      <c r="G26" s="31">
         <v>8.24</v>
       </c>
-      <c r="H26" s="46" t="s">
+      <c r="H26" s="30" t="s">
         <v>127</v>
       </c>
-      <c r="I26" s="46" t="s">
+      <c r="I26" s="30" t="s">
         <v>128</v>
       </c>
-      <c r="J26" s="46">
+      <c r="J26" s="30">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="K26" s="46" t="s">
+      <c r="K26" s="30" t="s">
         <v>129</v>
       </c>
-      <c r="L26" s="46">
+      <c r="L26" s="30">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="M26" s="46" t="s">
+      <c r="M26" s="30" t="s">
         <v>130</v>
       </c>
-      <c r="N26" s="46">
+      <c r="N26" s="30">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="O26" s="47">
+      <c r="O26" s="31">
         <v>32.96</v>
       </c>
-      <c r="P26" s="47">
+      <c r="P26" s="31">
         <v>46.9</v>
       </c>
-      <c r="Q26" s="47">
+      <c r="Q26" s="31">
         <v>45.84</v>
       </c>
     </row>
-    <row r="27" spans="2:18" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="53"/>
-      <c r="C27" s="49">
+    <row r="27" spans="2:17" ht="11.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="50"/>
+      <c r="C27" s="33">
         <v>68921</v>
       </c>
-      <c r="D27" s="49">
+      <c r="D27" s="33">
         <v>1467</v>
       </c>
-      <c r="E27" s="48">
+      <c r="E27" s="32">
         <v>27225</v>
       </c>
-      <c r="F27" s="50">
+      <c r="F27" s="34">
         <v>10.210000000000001</v>
       </c>
-      <c r="G27" s="50">
+      <c r="G27" s="34">
         <v>8.11</v>
       </c>
-      <c r="H27" s="49" t="s">
+      <c r="H27" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="I27" s="49" t="s">
+      <c r="I27" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="J27" s="49">
+      <c r="J27" s="33">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="K27" s="49" t="s">
+      <c r="K27" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="L27" s="49">
+      <c r="L27" s="33">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="M27" s="49" t="s">
+      <c r="M27" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="N27" s="49">
+      <c r="N27" s="33">
         <v>1.1000000000000001E-3</v>
       </c>
-      <c r="O27" s="50">
+      <c r="O27" s="34">
         <v>22.18</v>
       </c>
-      <c r="P27" s="50">
+      <c r="P27" s="34">
         <v>28.35</v>
       </c>
-      <c r="Q27" s="50">
+      <c r="Q27" s="34">
         <v>27.27</v>
       </c>
     </row>
-    <row r="28" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B28" s="56"/>
-    </row>
-    <row r="29" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B29" s="56"/>
+    <row r="28" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="B28" s="36"/>
+    </row>
+    <row r="29" spans="2:17" x14ac:dyDescent="0.2">
+      <c r="B29" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="M5:N5"/>
+    <mergeCell ref="O5:Q5"/>
     <mergeCell ref="B7:B17"/>
     <mergeCell ref="B19:B27"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="I5:J5"/>
     <mergeCell ref="K5:L5"/>
-    <mergeCell ref="M5:N5"/>
-    <mergeCell ref="O5:Q5"/>
   </mergeCells>
   <printOptions gridLines="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>